<commit_message>
Improve Mapping Output Consistency
</commit_message>
<xml_diff>
--- a/data/rules/mapping.xlsx
+++ b/data/rules/mapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/VV_Python_Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/VV_Python_Project/data/rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8C17B7-6CF4-1443-89F4-C9EDCF517C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7A4CC3B-8A3D-5840-AC49-4DB02D857D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="15380" windowWidth="24820" windowHeight="14060" xr2:uid="{03437215-B5EF-E446-BD16-C0E22245B470}"/>
+    <workbookView xWindow="4400" yWindow="680" windowWidth="28800" windowHeight="16480" xr2:uid="{03437215-B5EF-E446-BD16-C0E22245B470}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="236">
   <si>
     <t>Entity Type</t>
   </si>
@@ -1174,7 +1174,8 @@
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" customWidth="1"/>
     <col min="6" max="6" width="30.6640625" customWidth="1"/>
-    <col min="7" max="8" width="27.83203125" customWidth="1"/>
+    <col min="7" max="7" width="27.83203125" customWidth="1"/>
+    <col min="8" max="8" width="45.5" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
     <col min="10" max="10" width="45.83203125" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
@@ -3272,12 +3273,8 @@
       <c r="D73" s="2"/>
       <c r="E73" s="2"/>
       <c r="F73" s="2"/>
-      <c r="G73" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>119</v>
-      </c>
+      <c r="G73" s="1"/>
+      <c r="H73" s="1"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
       <c r="K73" s="7"/>

</xml_diff>